<commit_message>
Stock par chantier : colonnes RRS, SAR, PR et Code agent, nouvel ordre des colonnes
- RRS = Requestid du fichier LOGOPS ; SAR = QTE SAR et PR = Purchase Req. de l'État du stock
- Code agent (CODE AGT APPRO) remplace le code acheteur des commandes, dans le tableau et le contact des actions
- ordre : Statut, PN, CCN, RRS, À commander, Besoin, Stock, En cmd, SAR, PR, N° commande, PSD, Fournisseur,
  Code fournisseur, Action, Code agent, Gestion, TL, Date chantier (puis TRFX, Class code)
- besoin d'un PN demandé par plusieurs TRFX / RRS : additionné, TRFX et RRS listés
- données fictives et tests mis à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QT8GhHjeho8wXovFt7nryP
</commit_message>
<xml_diff>
--- a/tests/fixtures/besoins_chantier.xlsx
+++ b/tests/fixtures/besoins_chantier.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,6 +478,11 @@
           <t>Qty</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Requestid</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -503,6 +508,11 @@
       <c r="E4" t="n">
         <v>4</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>RRS-0001</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -528,16 +538,21 @@
       <c r="E5" t="n">
         <v>2</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>RRS-0002</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TRFX-02</t>
+          <t>TRFX-18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Housses</t>
+          <t>Housses arrière</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -553,6 +568,11 @@
       <c r="E6" t="n">
         <v>3</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>RRS-0003</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -578,6 +598,11 @@
       <c r="E7" t="n">
         <v>6</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>RRS-0004</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -603,6 +628,11 @@
       <c r="E8" t="n">
         <v>3</v>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>RRS-0005</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -628,6 +658,11 @@
       <c r="E9" t="n">
         <v>3</v>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>RRS-0006</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -653,6 +688,11 @@
       <c r="E10" t="n">
         <v>2</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>RRS-0007</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -678,6 +718,11 @@
       <c r="E11" t="n">
         <v>2</v>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>RRS-0008</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -703,6 +748,11 @@
       <c r="E12" t="n">
         <v>2</v>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>RRS-0009</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -728,6 +778,11 @@
       <c r="E13" t="n">
         <v>1</v>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>RRS-0010</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -753,6 +808,11 @@
       <c r="E14" t="n">
         <v>1</v>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>RRS-0011</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -778,6 +838,11 @@
       <c r="E15" t="n">
         <v>1</v>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>RRS-0012</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -803,6 +868,11 @@
       <c r="E16" t="n">
         <v>2</v>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>RRS-0013</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -828,6 +898,11 @@
       <c r="E17" t="n">
         <v>1</v>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>RRS-0014</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -851,6 +926,11 @@
       <c r="E18" t="n">
         <v>1</v>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>RRS-0015</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -876,6 +956,11 @@
       <c r="E19" t="n">
         <v>2</v>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>RRS-0016</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -901,6 +986,11 @@
       <c r="E20" t="n">
         <v>2</v>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>RRS-0017</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -920,6 +1010,11 @@
       </c>
       <c r="E21" t="n">
         <v>9</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>RRS-0018</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>